<commit_message>
﻿Phase 2 follow-up: customer name data, test plan, doc consolidation
- Customer name: add Name column to Customer_data; loader sets Customer.display_name;
  queries return it; resolve_identity uses the real name in greetings (was deriving a
  fake name from the email local-part). Verified end-to-end (greeting shows real name).
- Test plan: add docs/phase2-test-plan.md - 20 scenarios + 5 fact-checked per-customer
  scripts + standalone/flow/KB-regression cases + coverage matrix. Live run: 27/28
  correct (1 known generator deflection quirk on general KB-only queries, documented).
- Docs: consolidate phase2-kb-eval-set.md into phase2-test-plan.md (one test doc,
  no content lost); record Group C + item 18 as deliberately deferred; changelog updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/bfsi.xlsx
+++ b/data/bfsi.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="28.875" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -556,6 +556,11 @@
           <t>Country</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -596,6 +601,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Fathima Devasahayam</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -636,6 +646,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sayantini S</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -676,6 +691,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sireesha S</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -716,6 +736,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Digvijay Yadav</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -758,6 +783,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Suraj Golthi</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -800,6 +830,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Abhishek Jain</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -842,6 +877,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Nivethitha JM</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -884,6 +924,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Vikas Menon</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -926,6 +971,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Swati Nair</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -968,6 +1018,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Manish Desai</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1010,6 +1065,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Isha Rana</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1052,6 +1112,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Naveen Kapoor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1094,6 +1159,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Sneha Bhatt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1136,6 +1206,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Deepak Malhotra</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -1178,6 +1253,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Meera Iyer</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1220,6 +1300,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Sachin Trivedi</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -1262,6 +1347,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Tanya Saxena</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -1304,6 +1394,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Arvind Naik</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1346,6 +1441,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Shruti Reddy</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1388,6 +1488,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Yash Joshi</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -1430,6 +1535,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Lavanya Pandey</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -1470,6 +1580,11 @@
       <c r="H23" s="1" t="inlineStr">
         <is>
           <t>India</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Suresh Babu</t>
         </is>
       </c>
     </row>
@@ -11170,9 +11285,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>500000</v>
       </c>
@@ -11332,9 +11444,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>450000</v>
       </c>
@@ -11358,9 +11467,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>1000000</v>
       </c>
@@ -11452,9 +11558,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>350000</v>
       </c>
@@ -11478,9 +11581,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>300000</v>
       </c>
@@ -11572,9 +11672,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>1800000</v>
       </c>
@@ -11632,9 +11729,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>700000</v>
       </c>
@@ -11658,9 +11752,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
         <v>1500000</v>
       </c>
@@ -11718,9 +11809,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
         <v>400000</v>
       </c>
@@ -11880,9 +11968,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
         <v>550000</v>
       </c>
@@ -11940,9 +12025,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
         <v>1300000</v>
       </c>
@@ -11966,9 +12048,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
         <v>2000000</v>
       </c>
@@ -11992,9 +12071,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
         <v>650000</v>
       </c>
@@ -12018,9 +12094,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
         <v>600000</v>
       </c>
@@ -12112,9 +12185,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
         <v>500000</v>
       </c>
@@ -12138,9 +12208,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
         <v>1600000</v>
       </c>
@@ -12198,9 +12265,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
         <v>480000</v>
       </c>

</xml_diff>